<commit_message>
update RND week 18
</commit_message>
<xml_diff>
--- a/rates-nodispo/week-18/Analisis_Rates_NoDispo_7d.xlsx
+++ b/rates-nodispo/week-18/Analisis_Rates_NoDispo_7d.xlsx
@@ -20,23 +20,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Sev IPM" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · BajoRend" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Sin Conv" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Demanda NC" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Demanda No Convertida" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Por Corp" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Por Destino" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2C · Por País" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Sev ND" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Sev IPM" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · BajoRend" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Sin Conv" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Demanda NC" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Por Corp" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Por Destino" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta B2B Opaco · Por País" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Sev ND" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Sev IPM" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · BajoRend" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Sin Conv" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Demanda No Convertida" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Por Corp" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Por Destino" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta OP · Por País" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Sev ND" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Sev IPM" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · BajoRend" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Sin Conv" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Demanda NC" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Demanda No Convertida" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Por Corp" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Por Destino" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canasta CUG · Por País" sheetId="33" state="visible" r:id="rId33"/>
@@ -563,14 +563,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P80 · 18692 hoteles · target &lt;3%</t>
+          <t>P80 · 20016 hoteles · target &lt;3%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -608,10 +608,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.001658463513802696</v>
+        <v>0.001598721023181455</v>
       </c>
     </row>
     <row r="7">
@@ -626,10 +626,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.02193451744061631</v>
+        <v>0.02058353317346123</v>
       </c>
     </row>
     <row r="8">
@@ -644,10 +644,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>2034</v>
+        <v>2070</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.1088166060346672</v>
+        <v>0.1034172661870504</v>
       </c>
     </row>
     <row r="9">
@@ -662,10 +662,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1404</v>
+        <v>1520</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.07511234752835437</v>
+        <v>0.0759392486011191</v>
       </c>
     </row>
     <row r="10">
@@ -680,10 +680,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>14813</v>
+        <v>15982</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.7924780654825594</v>
+        <v>0.7984612310151878</v>
       </c>
     </row>
   </sheetData>
@@ -703,7 +703,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -723,7 +723,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
         <v>28</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.004339739615623063</v>
+        <v>0.004296455424274973</v>
       </c>
     </row>
     <row r="7">
@@ -782,7 +782,7 @@
         <v>226</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.03502789832610043</v>
+        <v>0.03467853306736228</v>
       </c>
     </row>
     <row r="8">
@@ -797,10 +797,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>950</v>
+        <v>971</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.1472411655300682</v>
+        <v>0.1489949363203928</v>
       </c>
     </row>
     <row r="9">
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.07796032238065716</v>
+        <v>0.07764308731011202</v>
       </c>
     </row>
     <row r="10">
@@ -833,10 +833,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>4745</v>
+        <v>4786</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.7354308741475512</v>
+        <v>0.7343869878778579</v>
       </c>
     </row>
   </sheetData>
@@ -876,7 +876,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -914,10 +914,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>5827</v>
+        <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.9031308121512709</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -932,10 +932,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>132</v>
+        <v>6002</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.02045877247365158</v>
+        <v>0.9209759091606567</v>
       </c>
     </row>
     <row r="8">
@@ -950,10 +950,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.02061376317420955</v>
+        <v>0.02056160810188737</v>
       </c>
     </row>
     <row r="9">
@@ -968,10 +968,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.02278363298202108</v>
+        <v>0.02301672548718735</v>
       </c>
     </row>
     <row r="10">
@@ -986,10 +986,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.03301301921884687</v>
+        <v>0.03544575725026853</v>
       </c>
     </row>
   </sheetData>
@@ -1037,7 +1037,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -5690,7 +5690,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8023,7 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8043,7 +8043,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
         <v>-114.2499999999998</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.06641728789635476</v>
+        <v>0.06641728789635475</v>
       </c>
       <c r="G25" s="16" t="n">
         <v>-15.35269129654919</v>
@@ -8918,7 +8918,7 @@
         <v>2278.94</v>
       </c>
       <c r="F29" s="14" t="n">
-        <v>0.06553750358113819</v>
+        <v>0.0655375035811382</v>
       </c>
       <c r="G29" s="16" t="n">
         <v>451.5186205317004</v>
@@ -9058,7 +9058,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="14" t="n">
-        <v>0.03071649846331387</v>
+        <v>0.03071649846331388</v>
       </c>
       <c r="G33" s="16" t="n">
         <v>0</v>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -9210,7 +9210,7 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9455,7 @@
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -9595,7 +9595,7 @@
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -9665,7 +9665,7 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -9866,7 +9866,7 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9886,7 +9886,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -10866,7 +10866,7 @@
         <v>6065.59</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>0.02500874661662356</v>
+        <v>0.02500874661662357</v>
       </c>
       <c r="G32" s="16" t="n">
         <v>422.1475259654633</v>
@@ -11403,7 +11403,7 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -11531,7 +11531,7 @@
         <v>5002.38</v>
       </c>
       <c r="F51" s="14" t="n">
-        <v>0.02768542912647766</v>
+        <v>0.02768542912647765</v>
       </c>
       <c r="G51" s="16" t="n">
         <v>596.7443993851685</v>
@@ -11698,7 +11698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11709,7 +11709,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11729,7 +11729,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -12231,7 +12231,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12371,7 +12371,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12406,7 +12406,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12581,7 +12581,7 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12651,7 +12651,7 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12826,7 +12826,7 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12896,7 +12896,7 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -12931,7 +12931,7 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13001,7 +13001,7 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13059,7 +13059,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>0.08471755571495086</v>
+        <v>0.08471755571495088</v>
       </c>
       <c r="G42" s="16" t="n">
         <v>0</v>
@@ -13071,7 +13071,7 @@
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13106,7 +13106,7 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13141,7 +13141,7 @@
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13176,7 +13176,7 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13281,7 +13281,7 @@
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13316,7 +13316,7 @@
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13351,7 +13351,7 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13421,7 +13421,7 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13561,7 +13561,7 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13596,7 +13596,7 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13631,7 +13631,7 @@
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13666,7 +13666,7 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13701,7 +13701,7 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13736,7 +13736,7 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13771,7 +13771,7 @@
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13806,7 +13806,7 @@
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13841,7 +13841,7 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13876,7 +13876,7 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13911,7 +13911,7 @@
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13946,7 +13946,7 @@
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -13981,7 +13981,7 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14004,7 +14004,7 @@
         <v>0</v>
       </c>
       <c r="F69" s="14" t="n">
-        <v>0.09765795669215852</v>
+        <v>0.0976579566921585</v>
       </c>
       <c r="G69" s="16" t="n">
         <v>0</v>
@@ -14016,7 +14016,7 @@
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14051,7 +14051,7 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14086,7 +14086,7 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14121,7 +14121,7 @@
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14156,7 +14156,7 @@
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14191,7 +14191,7 @@
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14226,7 +14226,7 @@
       </c>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14261,7 +14261,7 @@
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14296,7 +14296,7 @@
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14331,7 +14331,7 @@
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14366,7 +14366,7 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14401,7 +14401,7 @@
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14471,7 +14471,7 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14506,7 +14506,7 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14541,7 +14541,7 @@
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14576,7 +14576,7 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14611,7 +14611,7 @@
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14646,7 +14646,7 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14681,7 +14681,7 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14716,7 +14716,7 @@
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14751,7 +14751,7 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14786,7 +14786,7 @@
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14821,7 +14821,7 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14856,7 +14856,7 @@
       </c>
       <c r="I93" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14891,7 +14891,7 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14926,7 +14926,7 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14961,7 +14961,7 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -14996,7 +14996,7 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15031,7 +15031,7 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15066,7 +15066,7 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15101,7 +15101,7 @@
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15136,7 +15136,7 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15171,7 +15171,7 @@
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15206,7 +15206,7 @@
       </c>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15241,7 +15241,7 @@
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15276,7 +15276,7 @@
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15311,7 +15311,7 @@
       </c>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15346,7 +15346,7 @@
       </c>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15381,7 +15381,7 @@
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15416,7 +15416,7 @@
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15451,7 +15451,7 @@
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15486,7 +15486,7 @@
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15521,7 +15521,7 @@
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15556,7 +15556,7 @@
       </c>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15591,7 +15591,7 @@
       </c>
       <c r="I114" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15661,7 +15661,7 @@
       </c>
       <c r="I116" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15696,7 +15696,7 @@
       </c>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15731,7 +15731,7 @@
       </c>
       <c r="I118" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15766,7 +15766,7 @@
       </c>
       <c r="I119" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15801,7 +15801,7 @@
       </c>
       <c r="I120" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15836,7 +15836,7 @@
       </c>
       <c r="I121" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15871,7 +15871,7 @@
       </c>
       <c r="I122" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15906,7 +15906,7 @@
       </c>
       <c r="I123" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15941,7 +15941,7 @@
       </c>
       <c r="I124" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -15976,7 +15976,7 @@
       </c>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16011,7 +16011,7 @@
       </c>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16046,7 +16046,7 @@
       </c>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16081,7 +16081,7 @@
       </c>
       <c r="I128" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16116,7 +16116,7 @@
       </c>
       <c r="I129" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16151,7 +16151,7 @@
       </c>
       <c r="I130" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="I131" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16221,7 +16221,7 @@
       </c>
       <c r="I132" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16256,7 +16256,7 @@
       </c>
       <c r="I133" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16291,7 +16291,7 @@
       </c>
       <c r="I134" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16326,7 +16326,7 @@
       </c>
       <c r="I135" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="I136" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16396,7 +16396,7 @@
       </c>
       <c r="I137" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16431,7 +16431,7 @@
       </c>
       <c r="I138" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16466,7 +16466,7 @@
       </c>
       <c r="I139" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16501,7 +16501,7 @@
       </c>
       <c r="I140" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16536,7 +16536,7 @@
       </c>
       <c r="I141" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16571,7 +16571,7 @@
       </c>
       <c r="I142" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16606,7 +16606,7 @@
       </c>
       <c r="I143" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16641,7 +16641,7 @@
       </c>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16676,7 +16676,7 @@
       </c>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16711,7 +16711,7 @@
       </c>
       <c r="I146" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16746,7 +16746,7 @@
       </c>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16781,7 +16781,7 @@
       </c>
       <c r="I148" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16816,7 +16816,7 @@
       </c>
       <c r="I149" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16851,7 +16851,7 @@
       </c>
       <c r="I150" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16886,7 +16886,7 @@
       </c>
       <c r="I151" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16921,7 +16921,7 @@
       </c>
       <c r="I152" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16956,7 +16956,7 @@
       </c>
       <c r="I153" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -16991,7 +16991,7 @@
       </c>
       <c r="I154" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="I155" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17061,7 +17061,7 @@
       </c>
       <c r="I156" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17096,7 +17096,7 @@
       </c>
       <c r="I157" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17131,7 +17131,7 @@
       </c>
       <c r="I158" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17166,7 +17166,7 @@
       </c>
       <c r="I159" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17201,7 +17201,7 @@
       </c>
       <c r="I160" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17236,7 +17236,7 @@
       </c>
       <c r="I161" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17271,7 +17271,7 @@
       </c>
       <c r="I162" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17306,7 +17306,7 @@
       </c>
       <c r="I163" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17341,7 +17341,7 @@
       </c>
       <c r="I164" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17376,7 +17376,7 @@
       </c>
       <c r="I165" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17411,7 +17411,7 @@
       </c>
       <c r="I166" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17446,7 +17446,7 @@
       </c>
       <c r="I167" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17481,7 +17481,7 @@
       </c>
       <c r="I168" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="I169" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="I170" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17586,7 +17586,7 @@
       </c>
       <c r="I171" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17621,7 +17621,7 @@
       </c>
       <c r="I172" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C173" s="12" t="n">
@@ -17656,7 +17656,7 @@
       </c>
       <c r="I173" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17666,7 +17666,7 @@
       </c>
       <c r="B174" s="5" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="C174" s="12" t="n">
@@ -17691,7 +17691,7 @@
       </c>
       <c r="I174" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17726,7 +17726,42 @@
       </c>
       <c r="I175" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I176" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -17747,27 +17782,27 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Severity %NoDispo</t>
+          <t>Canasta OP · Severity %NoDispo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · P80 · target &lt;3%</t>
+          <t>B2B Opaco · P80 · target &lt;3%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -17808,7 +17843,7 @@
         <v>39</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.002361489554950046</v>
+        <v>0.002217925386715196</v>
       </c>
     </row>
     <row r="7">
@@ -17823,10 +17858,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.02125340599455041</v>
+        <v>0.02007506824385805</v>
       </c>
     </row>
     <row r="8">
@@ -17841,10 +17876,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1630</v>
+        <v>1635</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.098698153194066</v>
+        <v>0.09298225659690627</v>
       </c>
     </row>
     <row r="9">
@@ -17859,10 +17894,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1193</v>
+        <v>1214</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.0722373599757796</v>
+        <v>0.06904003639672429</v>
       </c>
     </row>
     <row r="10">
@@ -17877,10 +17912,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>13302</v>
+        <v>14343</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.805449591280654</v>
+        <v>0.8156847133757962</v>
       </c>
     </row>
   </sheetData>
@@ -17906,21 +17941,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Severity IPM (USD/M)</t>
+          <t>Canasta OP · Severity IPM (USD/M)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · P80 · target ≥ $650</t>
+          <t>B2B Opaco · P80 · target ≥ $650</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -17958,10 +17993,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>11680</v>
+        <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.7072358462004239</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -17976,10 +18011,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1046</v>
+        <v>13736</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.0633363608840448</v>
+        <v>0.781164695177434</v>
       </c>
     </row>
     <row r="8">
@@ -17994,10 +18029,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>985</v>
+        <v>1002</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.05964274901604602</v>
+        <v>0.05698362147406733</v>
       </c>
     </row>
     <row r="9">
@@ -18012,10 +18047,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1249</v>
+        <v>1287</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.07562821677263094</v>
+        <v>0.07319153776160145</v>
       </c>
     </row>
     <row r="10">
@@ -18030,10 +18065,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>1555</v>
+        <v>1559</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.09415682712685437</v>
+        <v>0.08866014558689718</v>
       </c>
     </row>
   </sheetData>
@@ -18066,14 +18101,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P80 · 18692 hoteles · target ≥ $650</t>
+          <t>P80 · 20016 hoteles · target ≥ $650</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -18111,10 +18146,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>11954</v>
+        <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.63952493045153</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -18129,10 +18164,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1706</v>
+        <v>14712</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.09126899208217419</v>
+        <v>0.7350119904076738</v>
       </c>
     </row>
     <row r="8">
@@ -18147,10 +18182,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1732</v>
+        <v>1824</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.09265996148084742</v>
+        <v>0.09112709832134293</v>
       </c>
     </row>
     <row r="9">
@@ -18165,10 +18200,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1684</v>
+        <v>1834</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.09009201797560454</v>
+        <v>0.09162669864108713</v>
       </c>
     </row>
     <row r="10">
@@ -18183,10 +18218,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>1616</v>
+        <v>1646</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.08645409800984379</v>
+        <v>0.08223421262989608</v>
       </c>
     </row>
   </sheetData>
@@ -18220,21 +18255,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Top 50 Bajo Rendimiento</t>
+          <t>Canasta OP · Top 50 Bajo Rendimiento</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · BKGS&gt;0 · ordenado por tráfico ↓</t>
+          <t>B2B Opaco · BKGS&gt;0 · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -20828,21 +20863,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Top 50 Sin Conversión</t>
+          <t>Canasta OP · Top 50 Sin Conversión</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · BKGS=0 · ordenado por tráfico ↓ · cohorte estructural</t>
+          <t>B2B Opaco · BKGS=0 · ordenado por tráfico ↓ · cohorte estructural</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -22873,21 +22908,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Top 50 Demanda No Convertida</t>
+          <t>Canasta OP · Top 50 Demanda No Convertida</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · tráfico × %NoDispo · ordenado por demanda perdida ↓</t>
+          <t>B2B Opaco · tráfico × %NoDispo · ordenado por demanda perdida ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -25217,7 +25252,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -25226,21 +25261,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Por Corporativo</t>
+          <t>Canasta OP · Por Corporativo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · Top 50 corp · ordenado por tráfico ↓</t>
+          <t>B2B Opaco · Top 50 corp · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -26255,7 +26290,7 @@
         <v>6650.84</v>
       </c>
       <c r="F33" s="14" t="n">
-        <v>0.01545218050279508</v>
+        <v>0.01545218050279509</v>
       </c>
       <c r="G33" s="16" t="n">
         <v>377.3979118628988</v>
@@ -26360,7 +26395,7 @@
         <v>1208.42</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>0.1170824743635684</v>
+        <v>0.1170824743635683</v>
       </c>
       <c r="G36" s="16" t="n">
         <v>88.56938116870511</v>
@@ -26955,7 +26990,7 @@
         <v>2530.29</v>
       </c>
       <c r="F53" s="14" t="n">
-        <v>0.004535477776961692</v>
+        <v>0.004535477776961693</v>
       </c>
       <c r="G53" s="16" t="n">
         <v>432.1950086343691</v>
@@ -27069,21 +27104,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Por Destino</t>
+          <t>Canasta OP · Por Destino</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · Top 50 destinos · ordenado por tráfico ↓</t>
+          <t>B2B Opaco · Top 50 destinos · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -28895,7 +28930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28906,27 +28941,27 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Canasta B2B Opaco · Por País</t>
+          <t>Canasta OP · Por País</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B2B (OP) · todos los países · ordenado por tráfico ↓</t>
+          <t>B2B Opaco · todos los países · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -30023,7 +30058,7 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -30688,7 +30723,7 @@
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -30758,7 +30793,7 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -30793,7 +30828,7 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -30863,7 +30898,7 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -30898,7 +30933,7 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -30933,7 +30968,7 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31108,7 +31143,7 @@
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31213,7 +31248,7 @@
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31283,7 +31318,7 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31388,7 +31423,7 @@
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31528,7 +31563,7 @@
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31563,7 +31598,7 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31598,7 +31633,7 @@
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31633,7 +31668,7 @@
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31668,7 +31703,7 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31703,7 +31738,7 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31738,7 +31773,7 @@
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31773,7 +31808,7 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31808,7 +31843,7 @@
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31843,7 +31878,7 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31878,7 +31913,7 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31948,7 +31983,7 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -31983,7 +32018,7 @@
       </c>
       <c r="I91" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32088,7 +32123,7 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32123,7 +32158,7 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32158,7 +32193,7 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32193,7 +32228,7 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32263,7 +32298,7 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32298,7 +32333,7 @@
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32333,7 +32368,7 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32368,7 +32403,7 @@
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32426,7 +32461,7 @@
         <v>0</v>
       </c>
       <c r="F104" s="14" t="n">
-        <v>0.02242348302729265</v>
+        <v>0.02242348302729266</v>
       </c>
       <c r="G104" s="16" t="n">
         <v>0</v>
@@ -32543,7 +32578,7 @@
       </c>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32578,7 +32613,7 @@
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32613,7 +32648,7 @@
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32683,7 +32718,7 @@
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32718,7 +32753,7 @@
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32788,7 +32823,7 @@
       </c>
       <c r="I114" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32823,7 +32858,7 @@
       </c>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32858,7 +32893,7 @@
       </c>
       <c r="I116" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32893,7 +32928,7 @@
       </c>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32928,7 +32963,7 @@
       </c>
       <c r="I118" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32963,7 +32998,7 @@
       </c>
       <c r="I119" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -32998,7 +33033,7 @@
       </c>
       <c r="I120" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33033,7 +33068,7 @@
       </c>
       <c r="I121" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33103,7 +33138,7 @@
       </c>
       <c r="I123" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33138,7 +33173,7 @@
       </c>
       <c r="I124" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33173,7 +33208,7 @@
       </c>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33208,7 +33243,7 @@
       </c>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33243,7 +33278,7 @@
       </c>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33278,7 +33313,7 @@
       </c>
       <c r="I128" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33301,7 +33336,7 @@
         <v>0</v>
       </c>
       <c r="F129" s="14" t="n">
-        <v>0.0839205103859544</v>
+        <v>0.08392051038595441</v>
       </c>
       <c r="G129" s="16" t="n">
         <v>0</v>
@@ -33313,7 +33348,7 @@
       </c>
       <c r="I129" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33348,7 +33383,7 @@
       </c>
       <c r="I130" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33418,7 @@
       </c>
       <c r="I131" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33418,7 +33453,7 @@
       </c>
       <c r="I132" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33453,7 +33488,7 @@
       </c>
       <c r="I133" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33488,7 +33523,7 @@
       </c>
       <c r="I134" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33523,7 +33558,7 @@
       </c>
       <c r="I135" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33558,7 +33593,7 @@
       </c>
       <c r="I136" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33593,7 +33628,7 @@
       </c>
       <c r="I137" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33628,7 +33663,7 @@
       </c>
       <c r="I138" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33663,7 +33698,7 @@
       </c>
       <c r="I139" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33698,7 +33733,7 @@
       </c>
       <c r="I140" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33768,7 +33803,7 @@
       </c>
       <c r="I142" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33803,7 +33838,7 @@
       </c>
       <c r="I143" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33838,7 +33873,7 @@
       </c>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33873,7 +33908,7 @@
       </c>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33908,7 +33943,7 @@
       </c>
       <c r="I146" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33943,7 +33978,7 @@
       </c>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -33978,7 +34013,7 @@
       </c>
       <c r="I148" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34048,7 +34083,7 @@
       </c>
       <c r="I150" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34083,7 +34118,7 @@
       </c>
       <c r="I151" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34118,7 +34153,7 @@
       </c>
       <c r="I152" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34153,7 +34188,7 @@
       </c>
       <c r="I153" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34188,7 +34223,7 @@
       </c>
       <c r="I154" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34223,7 +34258,7 @@
       </c>
       <c r="I155" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34258,7 +34293,7 @@
       </c>
       <c r="I156" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34293,7 +34328,7 @@
       </c>
       <c r="I157" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34328,7 +34363,7 @@
       </c>
       <c r="I158" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34363,7 +34398,7 @@
       </c>
       <c r="I159" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34398,7 +34433,7 @@
       </c>
       <c r="I160" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34433,7 +34468,7 @@
       </c>
       <c r="I161" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34468,7 +34503,7 @@
       </c>
       <c r="I162" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34503,7 +34538,7 @@
       </c>
       <c r="I163" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34538,7 +34573,7 @@
       </c>
       <c r="I164" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34573,7 +34608,7 @@
       </c>
       <c r="I165" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34608,7 +34643,7 @@
       </c>
       <c r="I166" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34643,7 +34678,7 @@
       </c>
       <c r="I167" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34678,7 +34713,7 @@
       </c>
       <c r="I168" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34713,7 +34748,7 @@
       </c>
       <c r="I169" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34748,7 +34783,7 @@
       </c>
       <c r="I170" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34783,7 +34818,7 @@
       </c>
       <c r="I171" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34818,7 +34853,7 @@
       </c>
       <c r="I172" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34853,7 +34888,7 @@
       </c>
       <c r="I173" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34888,7 +34923,7 @@
       </c>
       <c r="I174" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34923,7 +34958,42 @@
       </c>
       <c r="I175" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I176" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -34957,14 +35027,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · P80 · target &lt;3%</t>
+          <t>CUG · P80 · target &lt;3%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -35002,10 +35072,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.001343784994400896</v>
+        <v>0.001275142939410144</v>
       </c>
     </row>
     <row r="7">
@@ -35020,10 +35090,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.01773796192609182</v>
+        <v>0.01641232363950475</v>
       </c>
     </row>
     <row r="8">
@@ -35038,10 +35108,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1869</v>
+        <v>2013</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.08371780515117581</v>
+        <v>0.08280202377524577</v>
       </c>
     </row>
     <row r="9">
@@ -35056,10 +35126,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1429</v>
+        <v>1487</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.06400895856662935</v>
+        <v>0.06116572744848011</v>
       </c>
     </row>
     <row r="10">
@@ -35074,10 +35144,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>18601</v>
+        <v>20381</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.8331914893617022</v>
+        <v>0.8383447821973592</v>
       </c>
     </row>
   </sheetData>
@@ -35110,14 +35180,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · P80 · target ≥ $650</t>
+          <t>CUG · P80 · target ≥ $650</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -35155,10 +35225,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>17865</v>
+        <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.8002239641657335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -35173,10 +35243,10 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1062</v>
+        <v>20673</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.04756998880179171</v>
+        <v>0.8503558060137386</v>
       </c>
     </row>
     <row r="8">
@@ -35191,10 +35261,10 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>427</v>
+        <v>473</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.01912653975363942</v>
+        <v>0.01945621323680638</v>
       </c>
     </row>
     <row r="9">
@@ -35209,10 +35279,10 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>840</v>
+        <v>978</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.03762597984322508</v>
+        <v>0.04022870305622969</v>
       </c>
     </row>
     <row r="10">
@@ -35227,10 +35297,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>2131</v>
+        <v>2187</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.09545352743561031</v>
+        <v>0.08995927769322529</v>
       </c>
     </row>
   </sheetData>
@@ -35271,14 +35341,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · BKGS&gt;0 · ordenado por tráfico ↓</t>
+          <t>CUG · BKGS&gt;0 · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -37879,14 +37949,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · BKGS=0 · ordenado por tráfico ↓ · cohorte estructural</t>
+          <t>CUG · BKGS=0 · ordenado por tráfico ↓ · cohorte estructural</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -39932,7 +40002,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -40224,7 +40294,7 @@
         <v>-5251.93</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>0.2646688483495444</v>
+        <v>0.2646688483495443</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>-1121.798096292656</v>
@@ -40619,7 +40689,7 @@
         </is>
       </c>
       <c r="L18" s="12" t="n">
-        <v>995439.9999999999</v>
+        <v>995440</v>
       </c>
     </row>
     <row r="19">
@@ -40704,7 +40774,7 @@
         <v>12183.57</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>0.3076506690627428</v>
+        <v>0.3076506690627427</v>
       </c>
       <c r="J20" s="15" t="n">
         <v>4033.634895483983</v>
@@ -40715,7 +40785,7 @@
         </is>
       </c>
       <c r="L20" s="12" t="n">
-        <v>929257.0000000002</v>
+        <v>929257.0000000001</v>
       </c>
     </row>
     <row r="21">
@@ -40848,7 +40918,7 @@
         <v>16661.96</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>0.2043977109253355</v>
+        <v>0.2043977109253356</v>
       </c>
       <c r="J23" s="15" t="n">
         <v>4112.800907573081</v>
@@ -40859,7 +40929,7 @@
         </is>
       </c>
       <c r="L23" s="12" t="n">
-        <v>828065</v>
+        <v>828065.0000000001</v>
       </c>
     </row>
     <row r="24">
@@ -41099,7 +41169,7 @@
         </is>
       </c>
       <c r="L28" s="12" t="n">
-        <v>744701.9999999999</v>
+        <v>744702</v>
       </c>
     </row>
     <row r="29">
@@ -41147,7 +41217,7 @@
         </is>
       </c>
       <c r="L29" s="12" t="n">
-        <v>729191.9999999999</v>
+        <v>729192</v>
       </c>
     </row>
     <row r="30">
@@ -42435,14 +42505,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · tráfico × %NoDispo · ordenado por demanda perdida ↓</t>
+          <t>CUG · tráfico × %NoDispo · ordenado por demanda perdida ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -44775,7 +44845,7 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -44788,14 +44858,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · Top 50 corp · ordenado por tráfico ↓</t>
+          <t>CUG · Top 50 corp · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -45985,7 +46055,7 @@
         <v>22972.57</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>0.0138060554370632</v>
+        <v>0.01380605543706321</v>
       </c>
       <c r="G38" s="16" t="n">
         <v>2492.107671741196</v>
@@ -46020,7 +46090,7 @@
         <v>-3917.62</v>
       </c>
       <c r="F39" s="14" t="n">
-        <v>0.01237220616210537</v>
+        <v>0.01237220616210536</v>
       </c>
       <c r="G39" s="16" t="n">
         <v>-448.1121473391075</v>
@@ -46207,7 +46277,7 @@
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -46631,14 +46701,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · Top 50 destinos · ordenado por tráfico ↓</t>
+          <t>CUG · Top 50 destinos · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -47058,7 +47128,7 @@
         <v>132249.45</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.05027503091966413</v>
+        <v>0.05027503091966414</v>
       </c>
       <c r="G16" s="16" t="n">
         <v>1597.05849704831</v>
@@ -47863,7 +47933,7 @@
         <v>71302.23999999999</v>
       </c>
       <c r="F39" s="14" t="n">
-        <v>0.05482390586902029</v>
+        <v>0.05482390586902028</v>
       </c>
       <c r="G39" s="16" t="n">
         <v>2342.447665269028</v>
@@ -48450,7 +48520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48461,7 +48531,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -48474,14 +48544,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CUG (UOP) · todos los países · ordenado por tráfico ↓</t>
+          <t>CUG · todos los países · ordenado por tráfico ↓</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -50033,7 +50103,7 @@
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50208,7 +50278,7 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50278,7 +50348,7 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50313,7 +50383,7 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50348,7 +50418,7 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50453,7 +50523,7 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50593,7 +50663,7 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50663,7 +50733,7 @@
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50791,7 +50861,7 @@
         <v>0</v>
       </c>
       <c r="F70" s="14" t="n">
-        <v>0.02394806509505192</v>
+        <v>0.02394806509505193</v>
       </c>
       <c r="G70" s="16" t="n">
         <v>0</v>
@@ -50803,7 +50873,7 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50838,7 +50908,7 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -50896,7 +50966,7 @@
         <v>-404.21</v>
       </c>
       <c r="F73" s="14" t="n">
-        <v>0.02363224965867728</v>
+        <v>0.02363224965867727</v>
       </c>
       <c r="G73" s="16" t="n">
         <v>-484.9422090838634</v>
@@ -51048,7 +51118,7 @@
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51188,7 +51258,7 @@
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51223,7 +51293,7 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51258,7 +51328,7 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51328,7 +51398,7 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51363,7 +51433,7 @@
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51433,7 +51503,7 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51503,7 +51573,7 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51573,7 +51643,7 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51631,7 +51701,7 @@
         <v>0</v>
       </c>
       <c r="F94" s="14" t="n">
-        <v>0.005989277370389877</v>
+        <v>0.005989277370389876</v>
       </c>
       <c r="G94" s="16" t="n">
         <v>0</v>
@@ -51643,7 +51713,7 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51818,7 +51888,7 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51888,7 +51958,7 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -51981,7 +52051,7 @@
         <v>621.1</v>
       </c>
       <c r="F104" s="14" t="n">
-        <v>0.09683485707672723</v>
+        <v>0.09683485707672725</v>
       </c>
       <c r="G104" s="16" t="n">
         <v>1996.618189767131</v>
@@ -52028,7 +52098,7 @@
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52063,7 +52133,7 @@
       </c>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52098,7 +52168,7 @@
       </c>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52133,7 +52203,7 @@
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52168,7 +52238,7 @@
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52203,7 +52273,7 @@
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52238,7 +52308,7 @@
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52273,7 +52343,7 @@
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52308,7 +52378,7 @@
       </c>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52343,7 +52413,7 @@
       </c>
       <c r="I114" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52378,7 +52448,7 @@
       </c>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52448,7 +52518,7 @@
       </c>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52483,7 +52553,7 @@
       </c>
       <c r="I118" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52518,7 +52588,7 @@
       </c>
       <c r="I119" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52553,7 +52623,7 @@
       </c>
       <c r="I120" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52623,7 +52693,7 @@
       </c>
       <c r="I122" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52658,7 +52728,7 @@
       </c>
       <c r="I123" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52693,7 +52763,7 @@
       </c>
       <c r="I124" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52728,7 +52798,7 @@
       </c>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52763,7 +52833,7 @@
       </c>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52798,7 +52868,7 @@
       </c>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52833,7 +52903,7 @@
       </c>
       <c r="I128" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52868,7 +52938,7 @@
       </c>
       <c r="I129" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52903,7 +52973,7 @@
       </c>
       <c r="I130" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52938,7 +53008,7 @@
       </c>
       <c r="I131" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -52973,7 +53043,7 @@
       </c>
       <c r="I132" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53008,7 +53078,7 @@
       </c>
       <c r="I133" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53043,7 +53113,7 @@
       </c>
       <c r="I134" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53066,7 +53136,7 @@
         <v>0</v>
       </c>
       <c r="F135" s="14" t="n">
-        <v>0.1979078506381394</v>
+        <v>0.1979078506381395</v>
       </c>
       <c r="G135" s="16" t="n">
         <v>0</v>
@@ -53078,7 +53148,7 @@
       </c>
       <c r="I135" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53113,7 +53183,7 @@
       </c>
       <c r="I136" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53148,7 +53218,7 @@
       </c>
       <c r="I137" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53183,7 +53253,7 @@
       </c>
       <c r="I138" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53218,7 +53288,7 @@
       </c>
       <c r="I139" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53253,7 +53323,7 @@
       </c>
       <c r="I140" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53288,7 +53358,7 @@
       </c>
       <c r="I141" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53323,7 +53393,7 @@
       </c>
       <c r="I142" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53358,7 +53428,7 @@
       </c>
       <c r="I143" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53393,7 +53463,7 @@
       </c>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53428,7 +53498,7 @@
       </c>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53463,7 +53533,7 @@
       </c>
       <c r="I146" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53498,7 +53568,7 @@
       </c>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53533,7 +53603,7 @@
       </c>
       <c r="I148" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53568,7 +53638,7 @@
       </c>
       <c r="I149" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53603,7 +53673,7 @@
       </c>
       <c r="I150" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53638,7 +53708,7 @@
       </c>
       <c r="I151" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53673,7 +53743,7 @@
       </c>
       <c r="I152" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53743,7 +53813,7 @@
       </c>
       <c r="I154" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53778,7 +53848,7 @@
       </c>
       <c r="I155" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53813,7 +53883,7 @@
       </c>
       <c r="I156" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53848,7 +53918,7 @@
       </c>
       <c r="I157" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53883,7 +53953,7 @@
       </c>
       <c r="I158" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53918,7 +53988,7 @@
       </c>
       <c r="I159" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -53953,7 +54023,7 @@
       </c>
       <c r="I160" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54023,7 +54093,7 @@
       </c>
       <c r="I162" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54058,7 +54128,7 @@
       </c>
       <c r="I163" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54093,7 +54163,7 @@
       </c>
       <c r="I164" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54128,7 +54198,7 @@
       </c>
       <c r="I165" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54163,7 +54233,7 @@
       </c>
       <c r="I166" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54198,7 +54268,7 @@
       </c>
       <c r="I167" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54233,7 +54303,7 @@
       </c>
       <c r="I168" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54268,7 +54338,7 @@
       </c>
       <c r="I169" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54303,7 +54373,7 @@
       </c>
       <c r="I170" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54338,7 +54408,7 @@
       </c>
       <c r="I171" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54373,7 +54443,7 @@
       </c>
       <c r="I172" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54408,7 +54478,7 @@
       </c>
       <c r="I173" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54443,7 +54513,7 @@
       </c>
       <c r="I174" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54478,7 +54548,42 @@
       </c>
       <c r="I175" s="5" t="inlineStr">
         <is>
-          <t>Sin Conversión</t>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I176" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
         </is>
       </c>
     </row>
@@ -54526,7 +54631,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -55116,7 +55221,7 @@
         <v>209.55</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>0.004610105137645561</v>
+        <v>0.004610105137645562</v>
       </c>
       <c r="J17" s="15" t="n">
         <v>26.04884677758798</v>
@@ -55701,7 +55806,7 @@
         <v>-3503.83</v>
       </c>
       <c r="I30" s="14" t="n">
-        <v>0.006016334148688283</v>
+        <v>0.006016334148688285</v>
       </c>
       <c r="J30" s="15" t="n">
         <v>-507.7366944505629</v>
@@ -55881,7 +55986,7 @@
         <v>387.7699999999999</v>
       </c>
       <c r="I34" s="14" t="n">
-        <v>0.05205869796401383</v>
+        <v>0.05205869796401384</v>
       </c>
       <c r="J34" s="15" t="n">
         <v>57.56178053340948</v>
@@ -56878,7 +56983,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -57204,7 +57309,7 @@
         <v>5844174</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>0.03571539793305264</v>
+        <v>0.03571539793305265</v>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
@@ -57888,7 +57993,7 @@
         <v>4221754</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>0.06443080293167247</v>
+        <v>0.06443080293167248</v>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
@@ -58767,7 +58872,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -58947,7 +59052,7 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>5846</v>
+        <v>5845</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>1421356242</v>
@@ -59567,7 +59672,7 @@
         <v>143476.81</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>0.05172460609139643</v>
+        <v>0.05172460609139642</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>3172.531764939799</v>
@@ -60593,7 +60698,7 @@
         <v>15590.47</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>0.01534950778724655</v>
+        <v>0.01534950778724654</v>
       </c>
       <c r="H52" s="15" t="n">
         <v>1154.584160797399</v>
@@ -60766,7 +60871,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -62765,7 +62870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -62831,7 +62936,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>30008</v>
+        <v>30007</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>10040023613</v>
@@ -64761,7 +64866,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 05/05/2026 01:36 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 19:04 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -64825,7 +64930,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Escalar 31 hoteles Súper Críticos del P80 (%NoDispo &gt;60%)</t>
+          <t>Escalar 32 hoteles Súper Críticos del P80 (%NoDispo &gt;60%)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -64899,12 +65004,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Plan saneamiento 441 hoteles Crítica/Súper Crítica</t>
+          <t>Plan saneamiento 444 hoteles Crítica/Súper Crítica</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>220 migrados a Revisar</t>
+          <t>222 migrados a Revisar</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>